<commit_message>
docs: updated ui tests with further test cases
</commit_message>
<xml_diff>
--- a/docs/testing/ui/test_ui.xlsx
+++ b/docs/testing/ui/test_ui.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="68">
   <si>
     <t>Test</t>
   </si>
@@ -112,7 +112,7 @@
     <t>Register Responsiveness: Laptop</t>
   </si>
   <si>
-    <t>Register Responsiveness: Large Tablet</t>
+    <t>Register Responsiveness: Tablet</t>
   </si>
   <si>
     <t>Register Responsiveness: Large Phone</t>
@@ -136,13 +136,85 @@
     <t>Forgot Responsiveness: Laptop</t>
   </si>
   <si>
-    <t>Forgot Responsiveness: Large Tablet</t>
+    <t>Forgot Responsiveness: Tablet</t>
   </si>
   <si>
     <t>Forgot Responsiveness: Large Phone</t>
   </si>
   <si>
     <t>Forgot Responsiveness: Small Phone</t>
+  </si>
+  <si>
+    <t>Basket buttons</t>
+  </si>
+  <si>
+    <t>Basket Responsiveness: Large Desktop</t>
+  </si>
+  <si>
+    <t>Basket Responsiveness: Laptop</t>
+  </si>
+  <si>
+    <t>Basket Responsiveness: Tablet</t>
+  </si>
+  <si>
+    <t>Unnecesarry amount of whitespace but it's funcionally fine</t>
+  </si>
+  <si>
+    <t>Basket Responsiveness: Large Phone</t>
+  </si>
+  <si>
+    <t>In portrait mode, the item bubble's contents are weirdly positioned</t>
+  </si>
+  <si>
+    <t>Basket Responsiveness: Large Phone after fix</t>
+  </si>
+  <si>
+    <t>Basket Responsiveness: Small Phone</t>
+  </si>
+  <si>
+    <t>Basket Responsiveness: Large Desktop after fix</t>
+  </si>
+  <si>
+    <t>Basket Responsiveness: Laptop after fix</t>
+  </si>
+  <si>
+    <t>Basket Responsiveness: Tablet after fix</t>
+  </si>
+  <si>
+    <t>Profile buttons</t>
+  </si>
+  <si>
+    <t>Profile Responsiveness: Large Desktop</t>
+  </si>
+  <si>
+    <t>Profile Responsiveness: Laptop</t>
+  </si>
+  <si>
+    <t>Profile Responsiveness: Tablet</t>
+  </si>
+  <si>
+    <t>Profile Responsiveness: Large Phone</t>
+  </si>
+  <si>
+    <t>Profile Responsiveness: Small Phone</t>
+  </si>
+  <si>
+    <t>Admin buttons</t>
+  </si>
+  <si>
+    <t>Admin Responsiveness: Large Desktop</t>
+  </si>
+  <si>
+    <t>Admin Responsiveness: Laptop</t>
+  </si>
+  <si>
+    <t>Admin Responsiveness: Tablet</t>
+  </si>
+  <si>
+    <t>Admin Responsiveness: Large Phone</t>
+  </si>
+  <si>
+    <t>Admin Responsiveness: Small Phone</t>
   </si>
 </sst>
 </file>
@@ -323,7 +395,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E31" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E49" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="5">
     <tableColumn name="Test" id="1"/>
     <tableColumn name="Outcome" id="2"/>
@@ -949,132 +1021,366 @@
       <c r="E23" s="13"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="3"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="6"/>
+      <c r="A24" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" s="6">
+        <v>45985.0</v>
+      </c>
       <c r="E24" s="7"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="3"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="6"/>
+      <c r="A25" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" s="6">
+        <v>45985.0</v>
+      </c>
       <c r="E25" s="7"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="3"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="6"/>
+      <c r="A26" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="6">
+        <v>45985.0</v>
+      </c>
       <c r="E26" s="7"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="3"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="7"/>
+      <c r="A27" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="3"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="7"/>
+      <c r="A28" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="3"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="6"/>
+      <c r="A29" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" s="6">
+        <v>45985.0</v>
+      </c>
       <c r="E29" s="7"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="3"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="6"/>
+      <c r="A30" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" s="6">
+        <v>45985.0</v>
+      </c>
       <c r="E30" s="7"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="3"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="6"/>
+      <c r="A31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31" s="6">
+        <v>45985.0</v>
+      </c>
       <c r="E31" s="7"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="14"/>
-      <c r="E32" s="14"/>
+      <c r="A32" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E32" s="7"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="14"/>
-      <c r="E33" s="14"/>
+      <c r="A33" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" s="12">
+        <v>45985.0</v>
+      </c>
+      <c r="E33" s="13"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="14"/>
-      <c r="E34" s="14"/>
+      <c r="A34" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E34" s="7"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="14"/>
-      <c r="E35" s="14"/>
+      <c r="A35" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E35" s="7"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="14"/>
-      <c r="E36" s="14"/>
+      <c r="A36" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E36" s="7"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="14"/>
-      <c r="E37" s="14"/>
+      <c r="A37" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E37" s="7"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="14"/>
-      <c r="E38" s="14"/>
+      <c r="A38" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E38" s="7"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="14"/>
-      <c r="E39" s="14"/>
+      <c r="A39" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="12">
+        <v>45985.0</v>
+      </c>
+      <c r="E39" s="13"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="14"/>
-      <c r="E40" s="14"/>
+      <c r="A40" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E40" s="7"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="14"/>
-      <c r="E41" s="14"/>
+      <c r="A41" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E41" s="7"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="14"/>
-      <c r="E42" s="14"/>
+      <c r="A42" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E42" s="7"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="14"/>
-      <c r="E43" s="14"/>
+      <c r="A43" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E43" s="7"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="14"/>
-      <c r="E44" s="14"/>
+      <c r="A44" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44" s="6">
+        <v>45985.0</v>
+      </c>
+      <c r="E44" s="7"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="14"/>
-      <c r="E45" s="14"/>
+      <c r="A45" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B45" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C45" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D45" s="12">
+        <v>45985.0</v>
+      </c>
+      <c r="E45" s="13"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="14"/>
-      <c r="E46" s="14"/>
+      <c r="A46" s="3"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="5"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="7"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="14"/>
-      <c r="E47" s="14"/>
+      <c r="A47" s="3"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="5"/>
+      <c r="D47" s="6"/>
+      <c r="E47" s="7"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="14"/>
-      <c r="E48" s="14"/>
+      <c r="A48" s="3"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="6"/>
+      <c r="E48" s="7"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="14"/>
-      <c r="E49" s="14"/>
+      <c r="A49" s="3"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="6"/>
+      <c r="E49" s="7"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="14"/>
@@ -4892,22 +5198,26 @@
       <c r="A1003" s="14"/>
       <c r="E1003" s="14"/>
     </row>
+    <row r="1004" ht="15.75" customHeight="1">
+      <c r="A1004" s="14"/>
+      <c r="E1004" s="14"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B1:B1003">
+  <conditionalFormatting sqref="B1:B1004">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Success">
       <formula>NOT(ISERROR(SEARCH(("Success"),(B1))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:B1003">
+  <conditionalFormatting sqref="B1:B1004">
     <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH(("Fail"),(B1))))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B17 B19:B31">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B17 B19:B49">
       <formula1>"Success,Fail"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D2:D31">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D2:D49">
       <formula1>OR(NOT(ISERROR(DATEVALUE(D2))), AND(ISNUMBER(D2), LEFT(CELL("format", D2))="D"))</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B18">

</xml_diff>

<commit_message>
docs: updated ui tests with a comment
</commit_message>
<xml_diff>
--- a/docs/testing/ui/test_ui.xlsx
+++ b/docs/testing/ui/test_ui.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="82">
   <si>
     <t>Test</t>
   </si>
@@ -248,6 +248,9 @@
   </si>
   <si>
     <t>Item-List Responsiveness: Small Phone after fix</t>
+  </si>
+  <si>
+    <t>Price and amount are pushed into the border. Minimal problem but couldn't fix</t>
   </si>
   <si>
     <t>Item-List Responsiveness: Large Desktop after fix</t>
@@ -1543,11 +1546,13 @@
       <c r="D54" s="6">
         <v>45985.0</v>
       </c>
-      <c r="E54" s="14"/>
+      <c r="E54" s="15" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>6</v>
@@ -1562,7 +1567,7 @@
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B56" s="10" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
docs: updatet test_ui with test cases for edit
</commit_message>
<xml_diff>
--- a/docs/testing/ui/test_ui.xlsx
+++ b/docs/testing/ui/test_ui.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="88">
   <si>
     <t>Test</t>
   </si>
@@ -257,6 +257,24 @@
   </si>
   <si>
     <t>Item-List Responsiveness: Laptop after fix</t>
+  </si>
+  <si>
+    <t>Edit buttons</t>
+  </si>
+  <si>
+    <t>Edit Responsiveness: Large Desktop</t>
+  </si>
+  <si>
+    <t>Edit Responsiveness: Laptop</t>
+  </si>
+  <si>
+    <t>Edit Responsiveness: Tablet</t>
+  </si>
+  <si>
+    <t>Edit Responsiveness: Large Phone</t>
+  </si>
+  <si>
+    <t>Edit Responsiveness: Small Phone</t>
   </si>
 </sst>
 </file>
@@ -363,7 +381,7 @@
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1581,37 +1599,94 @@
       <c r="E56" s="16"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="17"/>
-      <c r="B57" s="4"/>
-      <c r="C57" s="5"/>
-      <c r="D57" s="6"/>
+      <c r="A57" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57" s="6">
+        <v>45988.0</v>
+      </c>
       <c r="E57" s="14"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="18"/>
-      <c r="B58" s="19"/>
-      <c r="D58" s="19"/>
-      <c r="E58" s="18"/>
+      <c r="A58" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D58" s="6">
+        <v>45988.0</v>
+      </c>
+      <c r="E58" s="14"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="18"/>
-      <c r="B59" s="19"/>
-      <c r="E59" s="18"/>
+      <c r="A59" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59" s="6">
+        <v>45988.0</v>
+      </c>
+      <c r="E59" s="14"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="18"/>
-      <c r="B60" s="19"/>
-      <c r="E60" s="18"/>
+      <c r="A60" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="6">
+        <v>45988.0</v>
+      </c>
+      <c r="E60" s="14"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="18"/>
-      <c r="B61" s="19"/>
-      <c r="E61" s="18"/>
+      <c r="A61" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D61" s="6">
+        <v>45988.0</v>
+      </c>
+      <c r="E61" s="14"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="18"/>
-      <c r="B62" s="19"/>
-      <c r="E62" s="18"/>
+      <c r="A62" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B62" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C62" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62" s="12">
+        <v>45988.0</v>
+      </c>
+      <c r="E62" s="16"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="18"/>
@@ -5394,10 +5469,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B17 B19:B57">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B17 B19:B62">
       <formula1>"Success,Fail"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D2:D57">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D2:D62">
       <formula1>OR(NOT(ISERROR(DATEVALUE(D2))), AND(ISNUMBER(D2), LEFT(CELL("format", D2))="D"))</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B18">

</xml_diff>

<commit_message>
docs: updated test ui with further test cases
</commit_message>
<xml_diff>
--- a/docs/testing/ui/test_ui.xlsx
+++ b/docs/testing/ui/test_ui.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="95">
   <si>
     <t>Test</t>
   </si>
@@ -293,15 +293,19 @@
   </si>
   <si>
     <t>Forgot Responsiveness: Small Phone after improvements</t>
+  </si>
+  <si>
+    <t>These are tests after the following improvements: removing placeholders, loading indicators, edit button, sidebar slide, and search</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy.MM.dd."/>
     <numFmt numFmtId="165" formatCode="yyyy.m.d."/>
+    <numFmt numFmtId="166" formatCode="yyyy.m.d"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -350,7 +354,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -417,6 +421,15 @@
     </xf>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -498,7 +511,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E68" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E80" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="5">
     <tableColumn name="Test" id="1"/>
     <tableColumn name="Outcome" id="2"/>
@@ -1809,52 +1822,186 @@
       <c r="E68" s="22"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="19"/>
-      <c r="E69" s="19"/>
+      <c r="A69" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D69" s="23">
+        <v>45990.0</v>
+      </c>
+      <c r="E69" s="24" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="19"/>
-      <c r="E70" s="19"/>
+      <c r="A70" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D70" s="23">
+        <v>45990.0</v>
+      </c>
+      <c r="E70" s="20"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="19"/>
-      <c r="E71" s="19"/>
+      <c r="A71" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C71" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" s="23">
+        <v>45990.0</v>
+      </c>
+      <c r="E71" s="20"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="19"/>
-      <c r="E72" s="19"/>
+      <c r="A72" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="23">
+        <v>45990.0</v>
+      </c>
+      <c r="E72" s="20"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="19"/>
-      <c r="E73" s="19"/>
+      <c r="A73" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73" s="23">
+        <v>45990.0</v>
+      </c>
+      <c r="E73" s="20"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="19"/>
-      <c r="E74" s="19"/>
+      <c r="A74" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B74" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C74" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74" s="25">
+        <v>45990.0</v>
+      </c>
+      <c r="E74" s="22"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="19"/>
-      <c r="E75" s="19"/>
+      <c r="A75" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C75" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D75" s="23">
+        <v>45990.0</v>
+      </c>
+      <c r="E75" s="20"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="19"/>
-      <c r="E76" s="19"/>
+      <c r="A76" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C76" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D76" s="23">
+        <v>45990.0</v>
+      </c>
+      <c r="E76" s="20"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="19"/>
-      <c r="E77" s="19"/>
+      <c r="A77" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D77" s="23">
+        <v>45990.0</v>
+      </c>
+      <c r="E77" s="20"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="19"/>
-      <c r="E78" s="19"/>
+      <c r="A78" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C78" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D78" s="23">
+        <v>45990.0</v>
+      </c>
+      <c r="E78" s="20"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="A79" s="19"/>
-      <c r="E79" s="19"/>
+      <c r="A79" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D79" s="23">
+        <v>45990.0</v>
+      </c>
+      <c r="E79" s="20"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="19"/>
-      <c r="E80" s="19"/>
+      <c r="A80" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B80" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C80" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D80" s="25">
+        <v>45990.0</v>
+      </c>
+      <c r="E80" s="22"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="19"/>
@@ -5564,7 +5711,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B17 B19:B62 B64:B68">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B17 B19:B62 B64:B80">
       <formula1>"Success,Fail"</formula1>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D2:D62">

</xml_diff>

<commit_message>
docs: updated ui tests with responsivness tests for chatbot
</commit_message>
<xml_diff>
--- a/docs/testing/ui/test_ui.xlsx
+++ b/docs/testing/ui/test_ui.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="96">
   <si>
     <t>Test</t>
   </si>
@@ -296,16 +296,20 @@
   </si>
   <si>
     <t>These are tests after the following improvements: removing placeholders, loading indicators, edit button, sidebar slide, and search</t>
+  </si>
+  <si>
+    <t>Chatbot Responsiveness</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy.MM.dd."/>
     <numFmt numFmtId="165" formatCode="yyyy.m.d."/>
     <numFmt numFmtId="166" formatCode="yyyy.m.d"/>
+    <numFmt numFmtId="167" formatCode="yyyy.mm.dd"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -354,7 +358,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -429,6 +433,21 @@
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="167" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -511,7 +530,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E80" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E86" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="5">
     <tableColumn name="Test" id="1"/>
     <tableColumn name="Outcome" id="2"/>
@@ -2004,28 +2023,86 @@
       <c r="E80" s="22"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
-      <c r="A81" s="19"/>
-      <c r="E81" s="19"/>
+      <c r="A81" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C81" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D81" s="26">
+        <v>45992.0</v>
+      </c>
+      <c r="E81" s="20"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
-      <c r="A82" s="19"/>
-      <c r="E82" s="19"/>
+      <c r="A82" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C82" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D82" s="26">
+        <v>45992.0</v>
+      </c>
+      <c r="E82" s="20"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
-      <c r="A83" s="19"/>
-      <c r="E83" s="19"/>
+      <c r="A83" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C83" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D83" s="26">
+        <v>45992.0</v>
+      </c>
+      <c r="E83" s="20"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
-      <c r="A84" s="19"/>
-      <c r="E84" s="19"/>
+      <c r="A84" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C84" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D84" s="26">
+        <v>45992.0</v>
+      </c>
+      <c r="E84" s="20"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="19"/>
-      <c r="E85" s="19"/>
+      <c r="A85" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B85" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C85" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D85" s="27">
+        <v>45992.0</v>
+      </c>
+      <c r="E85" s="22"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="19"/>
-      <c r="E86" s="19"/>
+      <c r="A86" s="28"/>
+      <c r="B86" s="29"/>
+      <c r="C86" s="5"/>
+      <c r="D86" s="30"/>
+      <c r="E86" s="20"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="19"/>
@@ -5711,7 +5788,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B17 B19:B62 B64:B80">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B17 B19:B62 B64:B85">
       <formula1>"Success,Fail"</formula1>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D2:D62">

</xml_diff>

<commit_message>
docs: updated ui tests with tests for modernized chatbot page
</commit_message>
<xml_diff>
--- a/docs/testing/ui/test_ui.xlsx
+++ b/docs/testing/ui/test_ui.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="105">
   <si>
     <t>Test</t>
   </si>
@@ -298,7 +298,34 @@
     <t>These are tests after the following improvements: removing placeholders, loading indicators, edit button, sidebar slide, and search</t>
   </si>
   <si>
-    <t>Chatbot Responsiveness</t>
+    <t>Chatbot Responsiveness: Large Desktop</t>
+  </si>
+  <si>
+    <t>Chatbot Responsiveness: Laptop</t>
+  </si>
+  <si>
+    <t>Chatbot Responsiveness: Tablet</t>
+  </si>
+  <si>
+    <t>Chatbot Responsiveness: Large Phone</t>
+  </si>
+  <si>
+    <t>Chatbot Responsiveness: Small Phone</t>
+  </si>
+  <si>
+    <t>Chatbot Responsiveness: Large Desktop after improvements</t>
+  </si>
+  <si>
+    <t>Chatbot Responsiveness: Laptop after improvement</t>
+  </si>
+  <si>
+    <t>Chatbot Responsiveness: Tablet after improvement</t>
+  </si>
+  <si>
+    <t>Chatbot Responsiveness: Large Phone after improvement</t>
+  </si>
+  <si>
+    <t>Chatbot Responsiveness: Small Phone after improvement</t>
   </si>
 </sst>
 </file>
@@ -358,7 +385,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="28">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -441,15 +468,6 @@
     <xf borderId="1" fillId="0" fontId="4" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -530,7 +548,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E86" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E90" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="5">
     <tableColumn name="Test" id="1"/>
     <tableColumn name="Outcome" id="2"/>
@@ -2039,7 +2057,7 @@
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>6</v>
@@ -2054,7 +2072,7 @@
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="15" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>6</v>
@@ -2069,7 +2087,7 @@
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="15" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>6</v>
@@ -2084,7 +2102,7 @@
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="17" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>6</v>
@@ -2098,27 +2116,79 @@
       <c r="E85" s="22"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="28"/>
-      <c r="B86" s="29"/>
-      <c r="C86" s="5"/>
-      <c r="D86" s="30"/>
+      <c r="A86" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C86" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D86" s="26">
+        <v>45992.0</v>
+      </c>
       <c r="E86" s="20"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
-      <c r="A87" s="19"/>
-      <c r="E87" s="19"/>
+      <c r="A87" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C87" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D87" s="26">
+        <v>45992.0</v>
+      </c>
+      <c r="E87" s="20"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
-      <c r="A88" s="19"/>
-      <c r="E88" s="19"/>
+      <c r="A88" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D88" s="26">
+        <v>45992.0</v>
+      </c>
+      <c r="E88" s="20"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
-      <c r="A89" s="19"/>
-      <c r="E89" s="19"/>
+      <c r="A89" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C89" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D89" s="26">
+        <v>45992.0</v>
+      </c>
+      <c r="E89" s="20"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
-      <c r="A90" s="19"/>
-      <c r="E90" s="19"/>
+      <c r="A90" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="B90" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C90" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D90" s="27">
+        <v>45992.0</v>
+      </c>
+      <c r="E90" s="22"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="19"/>
@@ -5788,7 +5858,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B17 B19:B62 B64:B85">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B17 B19:B62 B64:B90">
       <formula1>"Success,Fail"</formula1>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D2:D62">

</xml_diff>